<commit_message>
Added D2H endpoints for both models
</commit_message>
<xml_diff>
--- a/Random-Forest-main/Random Forest Data.xlsx
+++ b/Random-Forest-main/Random Forest Data.xlsx
@@ -1,22 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyliealfaro/Desktop/PhD UHM/Modeling Project/Random-Forest-main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A107EDDF-727D-EF4E-B196-BB7102EFBC69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CCA8776-0608-C142-9E08-999E3DFA4300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4360" yWindow="660" windowWidth="30200" windowHeight="21680" xr2:uid="{6AE4499B-BE9B-4430-8CBB-9E423EAAA4D3}"/>
+    <workbookView xWindow="3940" yWindow="660" windowWidth="30200" windowHeight="21680" xr2:uid="{6AE4499B-BE9B-4430-8CBB-9E423EAAA4D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Combined Manoa Data" sheetId="1" r:id="rId1"/>
     <sheet name="Hailey's Data" sheetId="3" r:id="rId2"/>
     <sheet name="Sheet1" sheetId="4" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Combined Manoa Data'!$B$2:$N$137</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -22183,6 +22186,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E174FB01-AC8B-4229-B319-63F7FF07E34C}">
+  <sheetPr filterMode="1"/>
   <dimension ref="B1:N148"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
@@ -22247,7 +22251,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="3" spans="2:14">
+    <row r="3" spans="2:14" hidden="1">
       <c r="B3" s="23">
         <v>44970.399305555555</v>
       </c>
@@ -22290,7 +22294,7 @@
         <v>-2.4</v>
       </c>
     </row>
-    <row r="4" spans="2:14">
+    <row r="4" spans="2:14" hidden="1">
       <c r="B4" s="23">
         <v>44970.429166666669</v>
       </c>
@@ -22419,7 +22423,7 @@
         <v>-5.0999999999999996</v>
       </c>
     </row>
-    <row r="7" spans="2:14">
+    <row r="7" spans="2:14" hidden="1">
       <c r="B7" s="23">
         <v>44974.370833333334</v>
       </c>
@@ -22462,7 +22466,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="8" spans="2:14">
+    <row r="8" spans="2:14" hidden="1">
       <c r="B8" s="23">
         <v>44974.385416666664</v>
       </c>
@@ -22505,7 +22509,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="9" spans="2:14">
+    <row r="9" spans="2:14" hidden="1">
       <c r="B9" s="23">
         <v>44974.432638888888</v>
       </c>
@@ -22548,7 +22552,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="10" spans="2:14">
+    <row r="10" spans="2:14" hidden="1">
       <c r="B10" s="23">
         <v>44977.37222222222</v>
       </c>
@@ -22591,7 +22595,7 @@
         <v>-3.6</v>
       </c>
     </row>
-    <row r="11" spans="2:14">
+    <row r="11" spans="2:14" hidden="1">
       <c r="B11" s="23">
         <v>44977.393055555556</v>
       </c>
@@ -22634,7 +22638,7 @@
         <v>-3.6</v>
       </c>
     </row>
-    <row r="12" spans="2:14">
+    <row r="12" spans="2:14" hidden="1">
       <c r="B12" s="23">
         <v>44977.43472222222</v>
       </c>
@@ -22677,7 +22681,7 @@
         <v>-3.6</v>
       </c>
     </row>
-    <row r="13" spans="2:14">
+    <row r="13" spans="2:14" hidden="1">
       <c r="B13" s="23">
         <v>44977.448611111111</v>
       </c>
@@ -22720,7 +22724,7 @@
         <v>-3.6</v>
       </c>
     </row>
-    <row r="14" spans="2:14">
+    <row r="14" spans="2:14" hidden="1">
       <c r="B14" s="23">
         <v>44979.367361111108</v>
       </c>
@@ -22763,7 +22767,7 @@
         <v>-3.8</v>
       </c>
     </row>
-    <row r="15" spans="2:14">
+    <row r="15" spans="2:14" hidden="1">
       <c r="B15" s="23">
         <v>44979.385416666664</v>
       </c>
@@ -22892,7 +22896,7 @@
         <v>-3.8</v>
       </c>
     </row>
-    <row r="18" spans="2:14">
+    <row r="18" spans="2:14" hidden="1">
       <c r="B18" s="23">
         <v>44981.361111111109</v>
       </c>
@@ -22935,7 +22939,7 @@
         <v>-3.1</v>
       </c>
     </row>
-    <row r="19" spans="2:14">
+    <row r="19" spans="2:14" hidden="1">
       <c r="B19" s="23">
         <v>44981.375</v>
       </c>
@@ -22978,7 +22982,7 @@
         <v>-3.1</v>
       </c>
     </row>
-    <row r="20" spans="2:14">
+    <row r="20" spans="2:14" hidden="1">
       <c r="B20" s="23">
         <v>44986.363888888889</v>
       </c>
@@ -23021,7 +23025,7 @@
         <v>-2.5</v>
       </c>
     </row>
-    <row r="21" spans="2:14">
+    <row r="21" spans="2:14" hidden="1">
       <c r="B21" s="23">
         <v>44986.381944444445</v>
       </c>
@@ -23064,7 +23068,7 @@
         <v>-2.5</v>
       </c>
     </row>
-    <row r="22" spans="2:14">
+    <row r="22" spans="2:14" hidden="1">
       <c r="B22" s="23">
         <v>44986.401388888888</v>
       </c>
@@ -23107,7 +23111,7 @@
         <v>-2.5</v>
       </c>
     </row>
-    <row r="23" spans="2:14">
+    <row r="23" spans="2:14" hidden="1">
       <c r="B23" s="23">
         <v>45019.381944444445</v>
       </c>
@@ -23150,7 +23154,7 @@
         <v>-3.7</v>
       </c>
     </row>
-    <row r="24" spans="2:14">
+    <row r="24" spans="2:14" hidden="1">
       <c r="B24" s="23">
         <v>45019.401388888888</v>
       </c>
@@ -23193,7 +23197,7 @@
         <v>-3.7</v>
       </c>
     </row>
-    <row r="25" spans="2:14">
+    <row r="25" spans="2:14" hidden="1">
       <c r="B25" s="23">
         <v>45028.354166666664</v>
       </c>
@@ -23236,7 +23240,7 @@
         <v>-2.6</v>
       </c>
     </row>
-    <row r="26" spans="2:14">
+    <row r="26" spans="2:14" hidden="1">
       <c r="B26" s="23">
         <v>45028.368750000001</v>
       </c>
@@ -23365,7 +23369,7 @@
         <v>-2.6</v>
       </c>
     </row>
-    <row r="29" spans="2:14">
+    <row r="29" spans="2:14" hidden="1">
       <c r="B29" s="23">
         <v>45033.361111111109</v>
       </c>
@@ -23408,7 +23412,7 @@
         <v>-1.5</v>
       </c>
     </row>
-    <row r="30" spans="2:14">
+    <row r="30" spans="2:14" hidden="1">
       <c r="B30" s="23">
         <v>45033.375</v>
       </c>
@@ -23451,7 +23455,7 @@
         <v>-1.5</v>
       </c>
     </row>
-    <row r="31" spans="2:14">
+    <row r="31" spans="2:14" hidden="1">
       <c r="B31" s="23">
         <v>45042.376388888886</v>
       </c>
@@ -23494,7 +23498,7 @@
         <v>-1.9</v>
       </c>
     </row>
-    <row r="32" spans="2:14">
+    <row r="32" spans="2:14" hidden="1">
       <c r="B32" s="23">
         <v>45058.451388888891</v>
       </c>
@@ -23537,7 +23541,7 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="33" spans="2:14">
+    <row r="33" spans="2:14" hidden="1">
       <c r="B33" s="23">
         <v>45061.423611111109</v>
       </c>
@@ -23666,7 +23670,7 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="36" spans="2:14">
+    <row r="36" spans="2:14" hidden="1">
       <c r="B36" s="23">
         <v>45061.486111111109</v>
       </c>
@@ -23709,7 +23713,7 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="37" spans="2:14">
+    <row r="37" spans="2:14" hidden="1">
       <c r="B37" s="23">
         <v>45062.475694444445</v>
       </c>
@@ -23752,7 +23756,7 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="38" spans="2:14">
+    <row r="38" spans="2:14" hidden="1">
       <c r="B38" s="23">
         <v>45062.489583333336</v>
       </c>
@@ -23795,7 +23799,7 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="39" spans="2:14">
+    <row r="39" spans="2:14" hidden="1">
       <c r="B39" s="23">
         <v>45062.53125</v>
       </c>
@@ -23838,7 +23842,7 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="40" spans="2:14">
+    <row r="40" spans="2:14" hidden="1">
       <c r="B40" s="23">
         <v>45063.464583333334</v>
       </c>
@@ -23881,7 +23885,7 @@
         <v>-1.3</v>
       </c>
     </row>
-    <row r="41" spans="2:14">
+    <row r="41" spans="2:14" hidden="1">
       <c r="B41" s="23">
         <v>45063.486111111109</v>
       </c>
@@ -23924,7 +23928,7 @@
         <v>-1.3</v>
       </c>
     </row>
-    <row r="42" spans="2:14">
+    <row r="42" spans="2:14" hidden="1">
       <c r="B42" s="23">
         <v>45077.625</v>
       </c>
@@ -23967,7 +23971,7 @@
         <v>-1.6</v>
       </c>
     </row>
-    <row r="43" spans="2:14">
+    <row r="43" spans="2:14" hidden="1">
       <c r="B43" s="23">
         <v>45077.635416666664</v>
       </c>
@@ -24096,7 +24100,7 @@
         <v>-1.6</v>
       </c>
     </row>
-    <row r="46" spans="2:14">
+    <row r="46" spans="2:14" hidden="1">
       <c r="B46" s="23">
         <v>45078.614583333336</v>
       </c>
@@ -24139,7 +24143,7 @@
         <v>-1.6</v>
       </c>
     </row>
-    <row r="47" spans="2:14">
+    <row r="47" spans="2:14" hidden="1">
       <c r="B47" s="23">
         <v>45078.627083333333</v>
       </c>
@@ -24182,7 +24186,7 @@
         <v>-1.6</v>
       </c>
     </row>
-    <row r="48" spans="2:14">
+    <row r="48" spans="2:14" hidden="1">
       <c r="B48" s="23">
         <v>45078.638194444444</v>
       </c>
@@ -24225,7 +24229,7 @@
         <v>-1.6</v>
       </c>
     </row>
-    <row r="49" spans="2:14">
+    <row r="49" spans="2:14" hidden="1">
       <c r="B49" s="23">
         <v>45079.39166666667</v>
       </c>
@@ -24268,7 +24272,7 @@
         <v>-1.6</v>
       </c>
     </row>
-    <row r="50" spans="2:14">
+    <row r="50" spans="2:14" hidden="1">
       <c r="B50" s="23">
         <v>45079.416666666664</v>
       </c>
@@ -24311,7 +24315,7 @@
         <v>-1.6</v>
       </c>
     </row>
-    <row r="51" spans="2:14">
+    <row r="51" spans="2:14" hidden="1">
       <c r="B51" s="23">
         <v>45121.4375</v>
       </c>
@@ -24354,7 +24358,7 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="52" spans="2:14">
+    <row r="52" spans="2:14" hidden="1">
       <c r="B52" s="23">
         <v>45121.458333333336</v>
       </c>
@@ -24440,7 +24444,7 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="54" spans="2:14">
+    <row r="54" spans="2:14" hidden="1">
       <c r="B54" s="23">
         <v>45124.368055555555</v>
       </c>
@@ -24483,7 +24487,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="55" spans="2:14">
+    <row r="55" spans="2:14" hidden="1">
       <c r="B55" s="23">
         <v>45124.375</v>
       </c>
@@ -24526,7 +24530,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="56" spans="2:14">
+    <row r="56" spans="2:14" hidden="1">
       <c r="B56" s="23">
         <v>45124.386805555558</v>
       </c>
@@ -24612,7 +24616,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="58" spans="2:14">
+    <row r="58" spans="2:14" hidden="1">
       <c r="B58" s="23">
         <v>45125.416666666664</v>
       </c>
@@ -24655,7 +24659,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="59" spans="2:14">
+    <row r="59" spans="2:14" hidden="1">
       <c r="B59" s="23">
         <v>45125.447916666664</v>
       </c>
@@ -24698,7 +24702,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="60" spans="2:14">
+    <row r="60" spans="2:14" hidden="1">
       <c r="B60" s="23">
         <v>45152.606249999997</v>
       </c>
@@ -24741,7 +24745,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="61" spans="2:14">
+    <row r="61" spans="2:14" hidden="1">
       <c r="B61" s="23">
         <v>45152.62222222222</v>
       </c>
@@ -24827,7 +24831,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="63" spans="2:14">
+    <row r="63" spans="2:14" hidden="1">
       <c r="B63" s="23">
         <v>45153.461805555555</v>
       </c>
@@ -24870,7 +24874,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="64" spans="2:14">
+    <row r="64" spans="2:14" hidden="1">
       <c r="B64" s="23">
         <v>45153.475694444445</v>
       </c>
@@ -24913,7 +24917,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="65" spans="2:14">
+    <row r="65" spans="2:14" hidden="1">
       <c r="B65" s="23">
         <v>45153.489583333336</v>
       </c>
@@ -24999,7 +25003,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="67" spans="2:14">
+    <row r="67" spans="2:14" hidden="1">
       <c r="B67" s="23">
         <v>45154.555555555555</v>
       </c>
@@ -25042,7 +25046,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="68" spans="2:14">
+    <row r="68" spans="2:14" hidden="1">
       <c r="B68" s="23">
         <v>45154.579861111109</v>
       </c>
@@ -25085,7 +25089,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="69" spans="2:14">
+    <row r="69" spans="2:14" hidden="1">
       <c r="B69" s="23">
         <v>45175.631944444445</v>
       </c>
@@ -25128,7 +25132,7 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="70" spans="2:14">
+    <row r="70" spans="2:14" hidden="1">
       <c r="B70" s="23">
         <v>45176.5625</v>
       </c>
@@ -25257,7 +25261,7 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="73" spans="2:14">
+    <row r="73" spans="2:14" hidden="1">
       <c r="B73" s="23">
         <v>45183.577777777777</v>
       </c>
@@ -25300,7 +25304,7 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="74" spans="2:14">
+    <row r="74" spans="2:14" hidden="1">
       <c r="B74" s="23">
         <v>45183.59375</v>
       </c>
@@ -25343,7 +25347,7 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="75" spans="2:14">
+    <row r="75" spans="2:14" hidden="1">
       <c r="B75" s="23">
         <v>45187.458333333336</v>
       </c>
@@ -25386,7 +25390,7 @@
         <v>-2.1</v>
       </c>
     </row>
-    <row r="76" spans="2:14">
+    <row r="76" spans="2:14" hidden="1">
       <c r="B76" s="23">
         <v>45187.474999999999</v>
       </c>
@@ -25429,7 +25433,7 @@
         <v>-2.1</v>
       </c>
     </row>
-    <row r="77" spans="2:14">
+    <row r="77" spans="2:14" hidden="1">
       <c r="B77" s="23">
         <v>45187.486805555556</v>
       </c>
@@ -25472,7 +25476,7 @@
         <v>-2.1</v>
       </c>
     </row>
-    <row r="78" spans="2:14">
+    <row r="78" spans="2:14" hidden="1">
       <c r="B78" s="23">
         <v>45238.506944444445</v>
       </c>
@@ -25515,7 +25519,7 @@
         <v>-1.5</v>
       </c>
     </row>
-    <row r="79" spans="2:14">
+    <row r="79" spans="2:14" hidden="1">
       <c r="B79" s="23">
         <v>45238.524305555555</v>
       </c>
@@ -25558,7 +25562,7 @@
         <v>-1.5</v>
       </c>
     </row>
-    <row r="80" spans="2:14">
+    <row r="80" spans="2:14" hidden="1">
       <c r="B80" s="23">
         <v>45238.546527777777</v>
       </c>
@@ -25687,7 +25691,7 @@
         <v>-1.5</v>
       </c>
     </row>
-    <row r="83" spans="2:14">
+    <row r="83" spans="2:14" hidden="1">
       <c r="B83" s="23">
         <v>45240.433333333334</v>
       </c>
@@ -25730,7 +25734,7 @@
         <v>-1.5</v>
       </c>
     </row>
-    <row r="84" spans="2:14">
+    <row r="84" spans="2:14" hidden="1">
       <c r="B84" s="23">
         <v>45240.462500000001</v>
       </c>
@@ -25773,7 +25777,7 @@
         <v>-1.5</v>
       </c>
     </row>
-    <row r="85" spans="2:14">
+    <row r="85" spans="2:14" hidden="1">
       <c r="B85" s="23">
         <v>45240.481944444444</v>
       </c>
@@ -25816,7 +25820,7 @@
         <v>-1.5</v>
       </c>
     </row>
-    <row r="86" spans="2:14">
+    <row r="86" spans="2:14" hidden="1">
       <c r="B86" s="23">
         <v>45240.5</v>
       </c>
@@ -25859,7 +25863,7 @@
         <v>-1.5</v>
       </c>
     </row>
-    <row r="87" spans="2:14">
+    <row r="87" spans="2:14" hidden="1">
       <c r="B87" s="23">
         <v>45259.463194444441</v>
       </c>
@@ -25902,7 +25906,7 @@
         <v>-2.8</v>
       </c>
     </row>
-    <row r="88" spans="2:14">
+    <row r="88" spans="2:14" hidden="1">
       <c r="B88" s="23">
         <v>45260.520833333336</v>
       </c>
@@ -26031,7 +26035,7 @@
         <v>-2.8</v>
       </c>
     </row>
-    <row r="91" spans="2:14">
+    <row r="91" spans="2:14" hidden="1">
       <c r="B91" s="23">
         <v>45260.590277777781</v>
       </c>
@@ -26074,7 +26078,7 @@
         <v>-2.8</v>
       </c>
     </row>
-    <row r="92" spans="2:14">
+    <row r="92" spans="2:14" hidden="1">
       <c r="B92" s="23">
         <v>45261.4375</v>
       </c>
@@ -26117,7 +26121,7 @@
         <v>-2.8</v>
       </c>
     </row>
-    <row r="93" spans="2:14">
+    <row r="93" spans="2:14" hidden="1">
       <c r="B93" s="23">
         <v>45261.45208333333</v>
       </c>
@@ -26160,7 +26164,7 @@
         <v>-2.8</v>
       </c>
     </row>
-    <row r="94" spans="2:14">
+    <row r="94" spans="2:14" hidden="1">
       <c r="B94" s="23">
         <v>45266.4375</v>
       </c>
@@ -26203,7 +26207,7 @@
         <v>-4.5999999999999996</v>
       </c>
     </row>
-    <row r="95" spans="2:14">
+    <row r="95" spans="2:14" hidden="1">
       <c r="B95" s="23">
         <v>45266.468055555553</v>
       </c>
@@ -26246,7 +26250,7 @@
         <v>-4.5999999999999996</v>
       </c>
     </row>
-    <row r="96" spans="2:14">
+    <row r="96" spans="2:14" hidden="1">
       <c r="B96" s="23">
         <v>45344.600694444445</v>
       </c>
@@ -26285,11 +26289,9 @@
       <c r="M96" s="19">
         <v>0.397368</v>
       </c>
-      <c r="N96" s="81">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="97" spans="2:14">
+      <c r="N96" s="81"/>
+    </row>
+    <row r="97" spans="2:14" hidden="1">
       <c r="B97" s="23">
         <v>45344.640277777777</v>
       </c>
@@ -26328,11 +26330,9 @@
       <c r="M97" s="19">
         <v>0.15940199999999999</v>
       </c>
-      <c r="N97" s="81">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98" spans="2:14">
+      <c r="N97" s="81"/>
+    </row>
+    <row r="98" spans="2:14" hidden="1">
       <c r="B98" s="23">
         <v>45344.663888888892</v>
       </c>
@@ -26371,11 +26371,9 @@
       <c r="M98" s="19">
         <v>5.8161600000000001E-2</v>
       </c>
-      <c r="N98" s="81">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99" spans="2:14">
+      <c r="N98" s="81"/>
+    </row>
+    <row r="99" spans="2:14" hidden="1">
       <c r="B99" s="23">
         <v>45344.681250000001</v>
       </c>
@@ -26414,9 +26412,7 @@
       <c r="M99" s="19">
         <v>0.16870099999999999</v>
       </c>
-      <c r="N99" s="81">
-        <v>0</v>
-      </c>
+      <c r="N99" s="81"/>
     </row>
     <row r="100" spans="2:14">
       <c r="B100" s="23">
@@ -26457,9 +26453,7 @@
       <c r="M100" s="19">
         <v>5.5910100000000004E-3</v>
       </c>
-      <c r="N100" s="81">
-        <v>0</v>
-      </c>
+      <c r="N100" s="81"/>
     </row>
     <row r="101" spans="2:14">
       <c r="B101" s="23">
@@ -26500,11 +26494,9 @@
       <c r="M101" s="19">
         <v>5.5910100000000004E-3</v>
       </c>
-      <c r="N101" s="81">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="102" spans="2:14">
+      <c r="N101" s="81"/>
+    </row>
+    <row r="102" spans="2:14" hidden="1">
       <c r="B102" s="23">
         <v>45351.558333333334</v>
       </c>
@@ -26543,11 +26535,9 @@
       <c r="M102" s="19">
         <v>2.23054E-2</v>
       </c>
-      <c r="N102" s="81">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" spans="2:14">
+      <c r="N102" s="81"/>
+    </row>
+    <row r="103" spans="2:14" hidden="1">
       <c r="B103" s="23">
         <v>45351.579861111109</v>
       </c>
@@ -26586,11 +26576,9 @@
       <c r="M103" s="19">
         <v>2.23054E-2</v>
       </c>
-      <c r="N103" s="81">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104" spans="2:14">
+      <c r="N103" s="81"/>
+    </row>
+    <row r="104" spans="2:14" hidden="1">
       <c r="B104" s="23">
         <v>45351.611805555556</v>
       </c>
@@ -26629,11 +26617,9 @@
       <c r="M104" s="19">
         <v>6.6970399999999999E-2</v>
       </c>
-      <c r="N104" s="81">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" spans="2:14">
+      <c r="N104" s="81"/>
+    </row>
+    <row r="105" spans="2:14" hidden="1">
       <c r="B105" s="26">
         <v>46001.361111111109</v>
       </c>
@@ -26675,7 +26661,7 @@
         <v>-1.4</v>
       </c>
     </row>
-    <row r="106" spans="2:14">
+    <row r="106" spans="2:14" hidden="1">
       <c r="B106" s="26">
         <v>46001.409722222219</v>
       </c>
@@ -26717,7 +26703,7 @@
         <v>-1.4</v>
       </c>
     </row>
-    <row r="107" spans="2:14">
+    <row r="107" spans="2:14" hidden="1">
       <c r="B107" s="26">
         <v>46001.473611111112</v>
       </c>
@@ -26759,7 +26745,7 @@
         <v>-1.4</v>
       </c>
     </row>
-    <row r="108" spans="2:14">
+    <row r="108" spans="2:14" hidden="1">
       <c r="B108" s="26">
         <v>46001.510416666664</v>
       </c>
@@ -26801,7 +26787,7 @@
         <v>-1.4</v>
       </c>
     </row>
-    <row r="109" spans="2:14">
+    <row r="109" spans="2:14" hidden="1">
       <c r="B109" s="26">
         <v>46001.536111111112</v>
       </c>
@@ -26885,7 +26871,7 @@
         <v>-1.4</v>
       </c>
     </row>
-    <row r="111" spans="2:14">
+    <row r="111" spans="2:14" hidden="1">
       <c r="B111" s="28">
         <v>46002</v>
       </c>
@@ -26928,7 +26914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="2:14">
+    <row r="112" spans="2:14" hidden="1">
       <c r="B112" s="28">
         <v>46002</v>
       </c>
@@ -26971,7 +26957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="2:14">
+    <row r="113" spans="2:14" hidden="1">
       <c r="B113" s="26">
         <v>46002.395833333336</v>
       </c>
@@ -27013,7 +26999,7 @@
         <v>-1.4</v>
       </c>
     </row>
-    <row r="114" spans="2:14">
+    <row r="114" spans="2:14" hidden="1">
       <c r="B114" s="28">
         <v>46022</v>
       </c>
@@ -27056,7 +27042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="2:14">
+    <row r="115" spans="2:14" hidden="1">
       <c r="B115" s="28">
         <v>46052</v>
       </c>
@@ -27099,7 +27085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="2:14">
+    <row r="116" spans="2:14" hidden="1">
       <c r="B116" s="28">
         <v>46056</v>
       </c>
@@ -27142,7 +27128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="2:14">
+    <row r="117" spans="2:14" hidden="1">
       <c r="B117" s="26">
         <v>46063.51458333333</v>
       </c>
@@ -27184,7 +27170,7 @@
         <v>-2.8</v>
       </c>
     </row>
-    <row r="118" spans="2:14">
+    <row r="118" spans="2:14" hidden="1">
       <c r="B118" s="26">
         <v>46063.522222222222</v>
       </c>
@@ -27226,7 +27212,7 @@
         <v>-2.8</v>
       </c>
     </row>
-    <row r="119" spans="2:14">
+    <row r="119" spans="2:14" hidden="1">
       <c r="B119" s="26">
         <v>46063.530555555553</v>
       </c>
@@ -27268,7 +27254,7 @@
         <v>-2.8</v>
       </c>
     </row>
-    <row r="120" spans="2:14">
+    <row r="120" spans="2:14" hidden="1">
       <c r="B120" s="26">
         <v>46063.538888888892</v>
       </c>
@@ -27352,7 +27338,7 @@
         <v>-2.8</v>
       </c>
     </row>
-    <row r="122" spans="2:14">
+    <row r="122" spans="2:14" hidden="1">
       <c r="B122" s="26">
         <v>46063.581944444442</v>
       </c>
@@ -27394,7 +27380,7 @@
         <v>-2.8</v>
       </c>
     </row>
-    <row r="123" spans="2:14">
+    <row r="123" spans="2:14" hidden="1">
       <c r="B123" s="28">
         <v>46065</v>
       </c>
@@ -27437,7 +27423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="2:14">
+    <row r="124" spans="2:14" hidden="1">
       <c r="B124" s="28">
         <v>46080</v>
       </c>
@@ -27480,7 +27466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="2:14">
+    <row r="125" spans="2:14" hidden="1">
       <c r="B125" s="28">
         <v>46093</v>
       </c>
@@ -27523,7 +27509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="2:14">
+    <row r="126" spans="2:14" hidden="1">
       <c r="B126" s="28">
         <v>46097</v>
       </c>
@@ -27566,7 +27552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="2:14">
+    <row r="127" spans="2:14" hidden="1">
       <c r="B127" s="26">
         <v>46105.353472222225</v>
       </c>
@@ -27608,7 +27594,7 @@
         <v>-6.4</v>
       </c>
     </row>
-    <row r="128" spans="2:14">
+    <row r="128" spans="2:14" hidden="1">
       <c r="B128" s="26">
         <v>46105.36041666667</v>
       </c>
@@ -27650,7 +27636,7 @@
         <v>-6.4</v>
       </c>
     </row>
-    <row r="129" spans="2:14">
+    <row r="129" spans="2:14" hidden="1">
       <c r="B129" s="26">
         <v>46105.366666666669</v>
       </c>
@@ -27692,7 +27678,7 @@
         <v>-6.4</v>
       </c>
     </row>
-    <row r="130" spans="2:14">
+    <row r="130" spans="2:14" hidden="1">
       <c r="B130" s="26">
         <v>46105.378472222219</v>
       </c>
@@ -27734,7 +27720,7 @@
         <v>-6.4</v>
       </c>
     </row>
-    <row r="131" spans="2:14">
+    <row r="131" spans="2:14" hidden="1">
       <c r="B131" s="28">
         <v>46112</v>
       </c>
@@ -27777,7 +27763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="2:14">
+    <row r="132" spans="2:14" hidden="1">
       <c r="B132" s="26">
         <v>46122.414583333331</v>
       </c>
@@ -27819,7 +27805,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="133" spans="2:14">
+    <row r="133" spans="2:14" hidden="1">
       <c r="B133" s="26">
         <v>46122.421527777777</v>
       </c>
@@ -27861,7 +27847,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="134" spans="2:14">
+    <row r="134" spans="2:14" hidden="1">
       <c r="B134" s="26">
         <v>46122.427777777775</v>
       </c>
@@ -27903,7 +27889,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="135" spans="2:14">
+    <row r="135" spans="2:14" hidden="1">
       <c r="B135" s="26">
         <v>46122.438888888886</v>
       </c>
@@ -27945,7 +27931,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="136" spans="2:14">
+    <row r="136" spans="2:14" hidden="1">
       <c r="B136" s="28">
         <v>46125</v>
       </c>
@@ -27989,7 +27975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="2:14" ht="17" thickBot="1">
+    <row r="137" spans="2:14" ht="17" hidden="1" thickBot="1">
       <c r="B137" s="37">
         <v>46142</v>
       </c>
@@ -28143,6 +28129,13 @@
       <c r="I148" s="18"/>
     </row>
   </sheetData>
+  <autoFilter ref="B2:N137" xr:uid="{E174FB01-AC8B-4229-B319-63F7FF07E34C}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="6"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:N148">
     <sortCondition ref="B1:B148"/>
   </sortState>

</xml_diff>